<commit_message>
Update exact warehouse staff count to 29 members across Financial Command Center
</commit_message>
<xml_diff>
--- a/warehouse_financial_system/BAO_CAO_TAI_CHINH_CHI_PHI_KHO.xlsx
+++ b/warehouse_financial_system/BAO_CAO_TAI_CHINH_CHI_PHI_KHO.xlsx
@@ -427,7 +427,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Thời gian lập báo cáo: 24/07/2026 17:56:14</t>
+          <t>Thời gian lập báo cáo: 24/07/2026 17:58:17</t>
         </is>
       </c>
     </row>
@@ -489,7 +489,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Quỹ lương 18 nhân sự kho (Bình quân 12,222,222 VND/người/tháng).</t>
+          <t>Quỹ lương 29 nhân sự kho (Bình quân 7,586,207 VND/người/tháng).</t>
         </is>
       </c>
     </row>
@@ -616,11 +616,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CHI PHÍ BÌNH QUÂN / 1 NHÂN SỰ KHO / THÁNG</t>
+          <t>CHI PHÍ BÌNH QUÂN / 1 NHÂN SỰ KHO / THÁNG (29 NGƯỜI)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>12222222</v>
+        <v>7586207</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -629,7 +629,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Quỹ lương chia cho 18 nhân sự</t>
+          <t>Quỹ lương chia cho 29 nhân sự kho thực tế</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 12h shift salary budget to 11.5M VND per person for 29 warehouse staff
</commit_message>
<xml_diff>
--- a/warehouse_financial_system/BAO_CAO_TAI_CHINH_CHI_PHI_KHO.xlsx
+++ b/warehouse_financial_system/BAO_CAO_TAI_CHINH_CHI_PHI_KHO.xlsx
@@ -420,14 +420,14 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>BÁO CÁO TỔNG HỢP CHI PHÍ VẬN HÀNH KHO &amp; P&amp;L THÁNG</t>
+          <t>BÁO CÁO TỔNG HỢP CHI PHÍ VẬN HÀNH KHO &amp; P&amp;L THÁNG (CA 12 HỜ)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Thời gian lập báo cáo: 24/07/2026 17:58:17</t>
+          <t>Thời gian lập báo cáo: 24/07/2026 17:59:53</t>
         </is>
       </c>
     </row>
@@ -464,7 +464,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>42.1%</t>
+          <t>34.0%</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -476,20 +476,20 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>⚡ 2. Chi Phí Nhân Công &amp; Nhặt Hàng</t>
+          <t>⚡ 2. Chi Phí Nhân Công (Ca 12 Tiếng)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>220000000</v>
+        <v>333500000</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>46.0%</t>
+          <t>56.4%</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Quỹ lương 29 nhân sự kho (Bình quân 7,586,207 VND/người/tháng).</t>
+          <t>Quỹ lương 29 nhân sự kho ca 12 tiếng (Bình quân 11,500,000 VND/người/tháng).</t>
         </is>
       </c>
     </row>
@@ -504,7 +504,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>3.8%</t>
+          <t>3.0%</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -524,7 +524,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>8.2%</t>
+          <t>6.6%</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -544,7 +544,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>47.8%</t>
+          <t>42.5%</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -560,7 +560,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>478000000</v>
+        <v>591500000</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -569,7 +569,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Tổng chi phí vận hành kho tháng</t>
+          <t>Tổng chi phí vận hành kho tháng (Lương ca 12h)</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5736000000</v>
+        <v>7098000000</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -616,11 +616,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CHI PHÍ BÌNH QUÂN / 1 NHÂN SỰ KHO / THÁNG (29 NGƯỜI)</t>
+          <t>CHI PHÍ BÌNH QUÂN / 1 NHÂN SỰ KHO CA 12H (29 NGƯỜI)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>7586207</v>
+        <v>11500000</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -629,7 +629,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Quỹ lương chia cho 29 nhân sự kho thực tế</t>
+          <t>Quỹ lương ca 12h chia cho 29 nhân sự kho (Bình quân 11.5 Tr/người)</t>
         </is>
       </c>
     </row>
@@ -660,7 +660,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>1062.22</v>
+        <v>1314.44</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1062.22</v>
+        <v>1314.44</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -726,7 +726,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>15933</v>
+        <v>19717</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -741,7 +741,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>531</v>
+        <v>657</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -756,7 +756,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>26556</v>
+        <v>32861</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -771,7 +771,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1275</v>
+        <v>1577</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -786,7 +786,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2124</v>
+        <v>2629</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -801,7 +801,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>850</v>
+        <v>1052</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -816,7 +816,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1062</v>
+        <v>1314</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -831,7 +831,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>53</v>
+        <v>66</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Update exact warehouse organizational salary structure (1 Manager @ 45M + 3 Storekeepers @ 20M + 25 Staff @ 10.5M = 367.5M VND)
</commit_message>
<xml_diff>
--- a/warehouse_financial_system/BAO_CAO_TAI_CHINH_CHI_PHI_KHO.xlsx
+++ b/warehouse_financial_system/BAO_CAO_TAI_CHINH_CHI_PHI_KHO.xlsx
@@ -414,260 +414,348 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>BÁO CÁO TỔNG HỢP CHI PHÍ VẬN HÀNH KHO &amp; P&amp;L THÁNG (CA 12 HỜ)</t>
+          <t>BÁO CÁO TỔNG HỢP CHI PHÍ VẬN HÀNH KHO &amp; P&amp;L THÁNG (CƠ CẤU LƯƠNG THỰC TẾ)</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Thời gian lập báo cáo: 24/07/2026 17:59:53</t>
+          <t>Thời gian lập báo cáo: 24/07/2026 18:01:29</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>HẠNG MỤC CHI PHÍ VẬN HÀNH KHO</t>
+          <t>CƠ CẤU LƯƠNG NHÂN SỰ KHO (29 NGƯỜI)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>CHI PHÍ THÁNG (VND)</t>
+          <t>SỐ LƯỢNG</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>% TRÊN TỔNG CHI PHÍ</t>
+          <t>MỨC LƯƠNG/NGƯỜI (VND)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>GHI CHÚ DIỄN GIẢI</t>
+          <t>TỔNG THÁNG (VND)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>🏗️ 1. Chi Phí Lưu Kho &amp; Hạ Tầng</t>
+          <t>1. Quản Lý Kho / Architect</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>201000000</v>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>34.0%</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Mặt bằng kho &amp; điện nước hạ tầng. Tính trên 4,038 vị trí (lấp đầy 94.1%).</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="C5" t="n">
+        <v>45000000</v>
+      </c>
+      <c r="D5" t="n">
+        <v>45000000</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>⚡ 2. Chi Phí Nhân Công (Ca 12 Tiếng)</t>
+          <t>2. Thủ Kho (Trưởng Ca)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>333500000</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>56.4%</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>Quỹ lương 29 nhân sự kho ca 12 tiếng (Bình quân 11,500,000 VND/người/tháng).</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="C6" t="n">
+        <v>20000000</v>
+      </c>
+      <c r="D6" t="n">
+        <v>60000000</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>📦 3. Chi Phí Vật Tư &amp; PE Quấn Pallet</t>
+          <t>3. Nhân Viên Kho Ca 12H</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>18000000</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>3.0%</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>Bao gồm màng PE quấn Pallet, băng keo, đai niềng, tem nhãn Barcode/QR.</t>
-        </is>
+        <v>25</v>
+      </c>
+      <c r="C7" t="n">
+        <v>10500000</v>
+      </c>
+      <c r="D7" t="n">
+        <v>262500000</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>🚜 4. Chi Phí Thiết Bị &amp; Xe Nâng</t>
+          <t>TỔNG QUỸ LƯƠNG NHÂN SỰ KHO</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>39000000</v>
+        <v>29</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>6.6%</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Khấu hao &amp; bảo trì 22 thiết bị IT, máy quét &amp; 4 Xe nâng hàng.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>📉 5. Chi Phí Giam Vốn Tồn Kho (Carrying Cost)</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>437500000</v>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>42.5%</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Chi phí cơ hội giam vốn (15.0%/năm trên 35.0 tỷ tồn kho).</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>367500000</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>HẠNG MỤC CHI PHÍ VẬN HÀNH KHO</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>CHI PHÍ THÁNG (VND)</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>% TRÊN TỔNG CHI PHÍ</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>GHI CHÚ DIỄN GIẢI</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>TỔNG CHI PHÍ OPEX KHO HÀNG THÁNG</t>
+          <t>🏗️ 1. Chi Phí Lưu Kho &amp; Hạ Tầng</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>591500000</v>
+        <v>201000000</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>100%</t>
+          <t>32.1%</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Tổng chi phí vận hành kho tháng (Lương ca 12h)</t>
+          <t>Mặt bằng kho &amp; điện nước hạ tầng. Tính trên 4,038 vị trí (lấp đầy 94.1%).</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>TỔNG CHI PHÍ OPEX KHO NĂM (DỰ TOÁN)</t>
+          <t>⚡ 2. Chi Phí Nhân Công (Cơ Cấu Thực Tế 29 Người)</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>7098000000</v>
+        <v>367500000</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>58.8%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Dự toán chi phí kho cả năm</t>
+          <t>Cơ cấu: 1 Quản lý kho (45Tr) + 3 Thủ kho (20Tr/người) + 25 Nhân viên ca 12h (10.5Tr/người).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>📦 3. Chi Phí Vật Tư &amp; PE Quấn Pallet</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>18000000</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2.9%</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Bao gồm màng PE quấn Pallet, băng keo, đai niềng, tem nhãn Barcode/QR.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>CHI PHÍ TRÊN 1 Ô KỆ / THÁNG (4,038 Ô KỆ)</t>
+          <t>🚜 4. Chi Phí Thiết Bị &amp; Xe Nâng</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>49777</v>
+        <v>39000000</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>VND/Ô Kệ</t>
+          <t>6.2%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Đơn giá ngày: 1,659 VND/ngày</t>
+          <t>Khấu hao &amp; bảo trì 22 thiết bị IT, máy quét &amp; 4 Xe nâng hàng.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CHI PHÍ BÌNH QUÂN / 1 NHÂN SỰ KHO CA 12H (29 NGƯỜI)</t>
+          <t>📉 5. Chi Phí Giam Vốn Tồn Kho (Carrying Cost)</t>
         </is>
       </c>
       <c r="B15" t="n">
-        <v>11500000</v>
+        <v>437500000</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>VND/Người</t>
+          <t>41.2%</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Quỹ lương ca 12h chia cho 29 nhân sự kho (Bình quân 11.5 Tr/người)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>CHI PHÍ BÌNH QUÂN / 1 THIẾT BỊ IT &amp; XE NÂNG</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>1772727</v>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>VND/Thiết bị</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>Chi phí bảo trì trên 22 thiết bị</t>
+          <t>Chi phí cơ hội giam vốn (15.0%/năm trên 35.0 tỷ tồn kho).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>TỔNG CHI PHÍ OPEX KHO HÀNG THÁNG</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>625500000</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>Tổng chi phí vận hành kho tháng</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>TỔNG CHI PHÍ OPEX KHO NĂM (DỰ TOÁN)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>7506000000</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Dự toán chi phí kho cả năm</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CHI PHÍ TRÊN 1 Ô KỆ / THÁNG (4,038 Ô KỆ)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>49777</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>VND/Ô Kệ</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>Đơn giá ngày: 1,659 VND/ngày</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>CHI PHÍ BÌNH QUÂN / 1 NHÂN SỰ KHO (29 NGƯỜI)</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>12672414</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>VND/Người</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Bình quân 12.67 Tr VND/người trên toàn bộ cơ cấu</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>CHI PHÍ BÌNH QUÂN / 1 THIẾT BỊ IT &amp; XE NÂNG</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>1772727</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>VND/Thiết bị</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Chi phí bảo trì trên 22 thiết bị</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
           <t>CHI PHÍ LƯU KHO &amp; XỬ LÝ TRÊN 1 KG</t>
         </is>
       </c>
-      <c r="B17" t="n">
-        <v>1314.44</v>
-      </c>
-      <c r="C17" t="inlineStr">
+      <c r="B23" t="n">
+        <v>1390</v>
+      </c>
+      <c r="C23" t="inlineStr">
         <is>
           <t>VND/Kg</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D23" t="inlineStr">
         <is>
           <t>Đơn giá bóc tách theo Kg</t>
         </is>
@@ -711,7 +799,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1314.44</v>
+        <v>1390</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -726,7 +814,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>19717</v>
+        <v>20850</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -741,7 +829,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>657</v>
+        <v>695</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -756,7 +844,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>32861</v>
+        <v>34750</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -771,7 +859,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1577</v>
+        <v>1668</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -786,7 +874,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2629</v>
+        <v>2780</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -801,7 +889,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1052</v>
+        <v>1112</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -816,7 +904,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1314</v>
+        <v>1390</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -831,7 +919,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Add Plastic Steel-Reinforced Pallet Fleet Depreciation & Loss Rate Engine (4,038 Pallets @ 1M VND) to Warehouse Financial System
</commit_message>
<xml_diff>
--- a/warehouse_financial_system/BAO_CAO_TAI_CHINH_CHI_PHI_KHO.xlsx
+++ b/warehouse_financial_system/BAO_CAO_TAI_CHINH_CHI_PHI_KHO.xlsx
@@ -414,348 +414,392 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>BÁO CÁO TỔNG HỢP CHI PHÍ VẬN HÀNH KHO &amp; P&amp;L THÁNG (CƠ CẤU LƯƠNG THỰC TẾ)</t>
+          <t>BÁO CÁO TỔNG HỢP CHI PHÍ VẬN HÀNH KHO &amp; KHẤU HAO/HAO HỤT PALLET NHỰA ỐNG SẮT</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Thời gian lập báo cáo: 24/07/2026 18:01:29</t>
+          <t>Thời gian lập báo cáo: 24/07/2026 18:07:24</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CƠ CẤU LƯƠNG NHÂN SỰ KHO (29 NGƯỜI)</t>
+          <t>BẢNG PHÂN TÍCH CHI PHÍ PALLET NHỰA ỐNG SẮT (1.000.000 VND/CÁI)</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SỐ LƯỢNG</t>
+          <t>CHỈ SỐ</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>MỨC LƯƠNG/NGƯỜI (VND)</t>
+          <t>GIÁ TRỊ THÁNG (VND)</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>TỔNG THÁNG (VND)</t>
+          <t>DIỄN GIẢI GIẢI TRÌNH</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>1. Quản Lý Kho / Architect</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" t="n">
-        <v>45000000</v>
-      </c>
-      <c r="D5" t="n">
-        <v>45000000</v>
+          <t>1. Tổng số lượng Pallet nhựa dẻo ống sắt trong kho</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>4,038 Pallet</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Phủ 4,032 ô kệ + 6 vùng đệm</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2. Thủ Kho (Trưởng Ca)</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>3</v>
-      </c>
-      <c r="C6" t="n">
-        <v>20000000</v>
-      </c>
-      <c r="D6" t="n">
-        <v>60000000</v>
+          <t>2. Tổng giá trị tài sản Pallet (1 Tr VND/Cái)</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>4,038,000,000 VND</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Vốn đầu tư ban đầu Pallet</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>3. Nhân Viên Kho Ca 12H</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>25</v>
-      </c>
-      <c r="C7" t="n">
-        <v>10500000</v>
-      </c>
-      <c r="D7" t="n">
-        <v>262500000</v>
+          <t>3. Chi phí Khấu hao Pallet (Khấu hao 5 năm)</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>67,300,000 VND</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Phân bổ 60 tháng</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>TỔNG QUỸ LƯƠNG NHÂN SỰ KHO</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>29</v>
+          <t>4. Chi phí Hao hụt / Gãy nứt / Bể Pallet (3%/Năm)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
+          <t>10,095,000 VND</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Dự phòng tổn thất xe nâng va chạm</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>TỔNG CHI PHÍ PALLET HÀNG THÁNG</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>367500000</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>HẠNG MỤC CHI PHÍ VẬN HÀNH KHO</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>CHI PHÍ THÁNG (VND)</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>% TRÊN TỔNG CHI PHÍ</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>GHI CHÚ DIỄN GIẢI</t>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>77,395,000 VND</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>Bình quân 19,167 VND/Pallet/tháng</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>🏗️ 1. Chi Phí Lưu Kho &amp; Hạ Tầng</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>201000000</v>
+          <t>HẠNG MỤC CHI PHÍ VẬN HÀNH KHO</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>CHI PHÍ THÁNG (VND)</t>
+        </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>32.1%</t>
+          <t>% TRÊN TỔNG CHI PHÍ</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Mặt bằng kho &amp; điện nước hạ tầng. Tính trên 4,038 vị trí (lấp đầy 94.1%).</t>
+          <t>GHI CHÚ DIỄN GIẢI</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>⚡ 2. Chi Phí Nhân Công (Cơ Cấu Thực Tế 29 Người)</t>
+          <t>🏗️ 1. Chi Phí Lưu Kho &amp; Hạ Tầng</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>367500000</v>
+        <v>201000000</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>58.8%</t>
+          <t>28.6%</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Cơ cấu: 1 Quản lý kho (45Tr) + 3 Thủ kho (20Tr/người) + 25 Nhân viên ca 12h (10.5Tr/người).</t>
+          <t>Mặt bằng kho &amp; điện nước hạ tầng. Tính trên 4,038 vị trí (lấp đầy 94.1%).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>📦 3. Chi Phí Vật Tư &amp; PE Quấn Pallet</t>
+          <t>⚡ 2. Chi Phí Nhân Công (Cơ Cấu Thực Tế 29 Người)</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>18000000</v>
+        <v>367500000</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.9%</t>
+          <t>52.3%</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Bao gồm màng PE quấn Pallet, băng keo, đai niềng, tem nhãn Barcode/QR.</t>
+          <t>Quỹ lương 29 người: 1 Quản lý (45Tr) + 3 Thủ kho (20Tr) + 25 Nhân viên ca 12h (10.5Tr).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>🚜 4. Chi Phí Thiết Bị &amp; Xe Nâng</t>
+          <t>📦 3. Chi Phí Vật Tư &amp; PE Quấn Pallet</t>
         </is>
       </c>
       <c r="B14" t="n">
-        <v>39000000</v>
+        <v>18000000</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>6.2%</t>
+          <t>2.6%</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Khấu hao &amp; bảo trì 22 thiết bị IT, máy quét &amp; 4 Xe nâng hàng.</t>
+          <t>Bao gồm màng PE quấn Pallet, băng keo, đai niềng, tem nhãn Barcode/QR.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>🚜 4. Chi Phí Xe Nâng &amp; Khấu Hao/Hao Hụt Pallet</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>116395000</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>16.6%</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Bảo trì xe nâng (25,000,000) + Khấu hao &amp; hao hụt 4,038 Pallet nhựa ống sắt (77,395,000 VND/tháng).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>📉 5. Chi Phí Giam Vốn Tồn Kho (Carrying Cost)</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B16" t="n">
         <v>437500000</v>
       </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>41.2%</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>38.4%</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
         <is>
           <t>Chi phí cơ hội giam vốn (15.0%/năm trên 35.0 tỷ tồn kho).</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>TỔNG CHI PHÍ OPEX KHO HÀNG THÁNG</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>625500000</v>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>100%</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>Tổng chi phí vận hành kho tháng</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>TỔNG CHI PHÍ OPEX KHO HÀNG THÁNG</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>702895000</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>Tổng chi phí vận hành kho tháng (Bao gồm Pallet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
           <t>TỔNG CHI PHÍ OPEX KHO NĂM (DỰ TOÁN)</t>
         </is>
       </c>
-      <c r="B18" t="n">
-        <v>7506000000</v>
-      </c>
-      <c r="C18" t="inlineStr">
+      <c r="B19" t="n">
+        <v>8434740000</v>
+      </c>
+      <c r="C19" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t>Dự toán chi phí kho cả năm</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>CHI PHÍ TRÊN 1 Ô KỆ / THÁNG (4,038 Ô KỆ)</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>49777</v>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>VND/Ô Kệ</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>Đơn giá ngày: 1,659 VND/ngày</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>CHI PHÍ BÌNH QUÂN / 1 NHÂN SỰ KHO (29 NGƯỜI)</t>
+          <t>CHI PHÍ TRÊN 1 Ô KỆ / THÁNG (4,038 Ô KỆ)</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>12672414</v>
+        <v>49777</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>VND/Người</t>
+          <t>VND/Ô Kệ</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Bình quân 12.67 Tr VND/người trên toàn bộ cơ cấu</t>
+          <t>Đơn giá ngày: 1,659 VND/ngày</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CHI PHÍ BÌNH QUÂN / 1 THIẾT BỊ IT &amp; XE NÂNG</t>
+          <t>CHI PHÍ BÌNH QUÂN / 1 NHÂN SỰ KHO (29 NGƯỜI)</t>
         </is>
       </c>
       <c r="B22" t="n">
-        <v>1772727</v>
+        <v>12672414</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>VND/Thiết bị</t>
+          <t>VND/Người</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Chi phí bảo trì trên 22 thiết bị</t>
+          <t>Bình quân 12.67 Tr VND/người trên toàn bộ cơ cấu</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>CHI PHÍ BÌNH QUÂN / 1 THIẾT BỊ IT &amp; XE NÂNG</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>5290682</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>VND/Thiết bị</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Chi phí bảo trì trên 22 thiết bị</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>CHI PHÍ LƯU KHO &amp; XỬ LÝ TRÊN 1 KG</t>
         </is>
       </c>
-      <c r="B23" t="n">
-        <v>1390</v>
-      </c>
-      <c r="C23" t="inlineStr">
+      <c r="B24" t="n">
+        <v>1561.99</v>
+      </c>
+      <c r="C24" t="inlineStr">
         <is>
           <t>VND/Kg</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>Đơn giá bóc tách theo Kg</t>
         </is>
@@ -799,7 +843,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1390</v>
+        <v>1561.99</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -814,7 +858,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>20850</v>
+        <v>23430</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -829,7 +873,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>695</v>
+        <v>781</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -844,7 +888,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>34750</v>
+        <v>39050</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -859,7 +903,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1668</v>
+        <v>1874</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -874,7 +918,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>2780</v>
+        <v>3124</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -889,7 +933,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>1112</v>
+        <v>1250</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -904,7 +948,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>1390</v>
+        <v>1562</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -919,7 +963,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>

</xml_diff>